<commit_message>
Dash Risco - 2026-05-04
</commit_message>
<xml_diff>
--- a/Dados/FechamentoNTNBs.xlsx
+++ b/Dados/FechamentoNTNBs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Asset Management\Equipe\Emanuel\21.0-Risco\DashRisco\Dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Asset Management\Equipe\Marcos\Risco\Projeto-Gestao-Risco\Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{402A344C-7204-46DD-88DB-0331D4E98FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C166A0-DBD6-448B-BA8F-8B3A51EA39ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="910" yWindow="980" windowWidth="28800" windowHeight="15360" xr2:uid="{463535B5-4209-4E39-8A9D-1F2BF9A6496F}"/>
+    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{463535B5-4209-4E39-8A9D-1F2BF9A6496F}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha2" sheetId="2" r:id="rId1"/>
@@ -54,21 +54,10 @@
     <definedName name="_ECO_RANGE_IDf639647b9bcc48079d4088b8fcffd216" localSheetId="0" hidden="1">Planilha2!$E$4:$E$205</definedName>
     <definedName name="_ECO_RANGE_IDfded19ac61144328a3001e7c39cb8209" localSheetId="0" hidden="1">Planilha2!$K$4:$K$205</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -153,9 +142,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -185,10 +171,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -206,185 +191,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
-<volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <volType type="realTimeData">
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a637ac45-155c-4eb1-909b-9892971d3578</stp>
-        <tr r="D3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>b619a35e-7cf3-4000-8fb9-35d4e393809a</stp>
-        <tr r="F3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>d4097a7e-3148-49f0-ac91-f9081f5b6e2c</stp>
-        <tr r="E3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>46d6068c-aef8-44d7-8b62-ff9286bdad69</stp>
-        <tr r="I3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>fd3f09ab-5019-40b9-93da-664184f1ae6b</stp>
-        <tr r="H3" s="1"/>
-      </tp>
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>fcb460ea-2975-461b-83f1-9f5d27b98e6c</stp>
-        <tr r="J3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>98368a77-d558-4bfd-9ebc-b6c7f5294f8c</stp>
-        <tr r="F3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b83d68fc-f616-4515-bb1a-3991e14e4629</stp>
-        <tr r="K3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>84798e3b-8833-4fc0-9428-688268c8b7d6</stp>
-        <tr r="L3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>73745083-0054-4052-aee0-f1ddd699f888</stp>
-        <tr r="C3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>2ade9665-e203-421e-8e5a-dd58ffb3eed1</stp>
-        <tr r="A3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>14d563c5-5871-42ee-95cb-dc6436419e65</stp>
-        <tr r="K3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>a768c611-16c2-4c59-9188-4e705b6c220a</stp>
-        <tr r="A3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>86b2b1de-230a-48df-9cd5-4371e43753fd</stp>
-        <tr r="H3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>d5463b85-f23a-49a6-afb1-6f0fd4d08495</stp>
-        <tr r="J3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>3c2da92a-e704-46f4-a851-c96d8453d1dc</stp>
-        <tr r="D3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>79e27e29-05ea-493e-b064-95d962094904</stp>
-        <tr r="G3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>41ea4885-40d1-4165-ba6f-716864d3257a</stp>
-        <tr r="G3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>b4abd981-9f2a-4c9a-914a-7af7c5f189ce</stp>
-        <tr r="E3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>d2e37414-13c4-4096-b2e7-bc5805a0f8a4</stp>
-        <tr r="C3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>c4e84715-9002-4d63-9c6c-ba681fe672ff</stp>
-        <tr r="L3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_670d653a32df4539babd0b6b70e689ad">
-      <tp>
-        <v>2</v>
-        <stp/>
-        <stp>a5bd3c93-755c-49b2-969e-a77cac8aa676</stp>
-        <tr r="I3" s="2"/>
-      </tp>
-    </main>
-  </volType>
-</volTypes>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -422,7 +232,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -528,7 +338,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -670,7 +480,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -679,12 +489,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33FBCE06-A615-4263-8DE6-4D9EB2327E61}">
   <dimension ref="A1:L205"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -722,7 +532,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -760,53 +570,53 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="2">
-        <f>_xll.ECONOMATICA(B1,"YTM",,"D-0","2025-01-01","D",,,,"FALSE",,)</f>
-        <v>45658</v>
-      </c>
-      <c r="C3" t="str">
-        <f>_xll.ECONOMATICA(C1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <f>_xll.ECONOMATICA(D1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <f>_xll.ECONOMATICA(E1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <f>_xll.ECONOMATICA(F1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <f>_xll.ECONOMATICA(G1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <f>_xll.ECONOMATICA(H1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <f>_xll.ECONOMATICA(I1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <f>_xll.ECONOMATICA(J1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="K3" t="str">
-        <f>_xll.ECONOMATICA(K1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <f>_xll.ECONOMATICA(L1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="e">
+        <f ca="1">_xll.ECONOMATICA(B1,"YTM",,"D-0","2025-01-01","D",,,,"FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="C3" t="e">
+        <f ca="1">_xll.ECONOMATICA(C1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="D3" t="e">
+        <f ca="1">_xll.ECONOMATICA(D1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="E3" t="e">
+        <f ca="1">_xll.ECONOMATICA(E1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="F3" t="e">
+        <f ca="1">_xll.ECONOMATICA(F1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="G3" t="e">
+        <f ca="1">_xll.ECONOMATICA(G1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="H3" t="e">
+        <f ca="1">_xll.ECONOMATICA(H1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I3" t="e">
+        <f ca="1">_xll.ECONOMATICA(I1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J3" t="e">
+        <f ca="1">_xll.ECONOMATICA(J1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="K3" t="e">
+        <f ca="1">_xll.ECONOMATICA(K1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="L3" t="e">
+        <f ca="1">_xll.ECONOMATICA(L1,"YTM",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>45659</v>
       </c>
@@ -844,7 +654,7 @@
         <v>7.3925999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>45660</v>
       </c>
@@ -882,7 +692,7 @@
         <v>7.3712</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>45663</v>
       </c>
@@ -920,7 +730,7 @@
         <v>7.3220999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>45664</v>
       </c>
@@ -958,7 +768,7 @@
         <v>7.3197999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>45665</v>
       </c>
@@ -996,7 +806,7 @@
         <v>7.3102</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>45666</v>
       </c>
@@ -1034,7 +844,7 @@
         <v>7.3236999999999997</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>45667</v>
       </c>
@@ -1072,7 +882,7 @@
         <v>7.3765000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>45670</v>
       </c>
@@ -1110,7 +920,7 @@
         <v>7.4173999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>45671</v>
       </c>
@@ -1148,7 +958,7 @@
         <v>7.3796999999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>45672</v>
       </c>
@@ -1186,7 +996,7 @@
         <v>7.3381999999999996</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>45673</v>
       </c>
@@ -1224,7 +1034,7 @@
         <v>7.39</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>45674</v>
       </c>
@@ -1262,7 +1072,7 @@
         <v>7.4725999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>45677</v>
       </c>
@@ -1300,7 +1110,7 @@
         <v>7.5232999999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>45678</v>
       </c>
@@ -1338,7 +1148,7 @@
         <v>7.5747999999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>45679</v>
       </c>
@@ -1376,7 +1186,7 @@
         <v>7.5625</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>45680</v>
       </c>
@@ -1414,7 +1224,7 @@
         <v>7.6021999999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>45681</v>
       </c>
@@ -1452,7 +1262,7 @@
         <v>7.5891999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>45684</v>
       </c>
@@ -1490,7 +1300,7 @@
         <v>7.5892999999999997</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>45685</v>
       </c>
@@ -1528,7 +1338,7 @@
         <v>7.5976999999999997</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>45686</v>
       </c>
@@ -1566,7 +1376,7 @@
         <v>7.6035000000000004</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>45687</v>
       </c>
@@ -1604,7 +1414,7 @@
         <v>7.4682000000000004</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>45688</v>
       </c>
@@ -1642,7 +1452,7 @@
         <v>7.4941000000000004</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>45691</v>
       </c>
@@ -1680,7 +1490,7 @@
         <v>7.4527999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>45692</v>
       </c>
@@ -1718,7 +1528,7 @@
         <v>7.4653</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>45693</v>
       </c>
@@ -1756,7 +1566,7 @@
         <v>7.5335000000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>45694</v>
       </c>
@@ -1794,7 +1604,7 @@
         <v>7.4932999999999996</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>45695</v>
       </c>
@@ -1832,7 +1642,7 @@
         <v>7.5236000000000001</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>45698</v>
       </c>
@@ -1870,7 +1680,7 @@
         <v>7.5218999999999996</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>45699</v>
       </c>
@@ -1908,7 +1718,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>45700</v>
       </c>
@@ -1946,7 +1756,7 @@
         <v>7.4949000000000003</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>45701</v>
       </c>
@@ -1984,7 +1794,7 @@
         <v>7.4817</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>45702</v>
       </c>
@@ -2022,7 +1832,7 @@
         <v>7.3483000000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>45705</v>
       </c>
@@ -2060,7 +1870,7 @@
         <v>7.3048000000000002</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>45706</v>
       </c>
@@ -2098,7 +1908,7 @@
         <v>7.3183999999999996</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>45707</v>
       </c>
@@ -2136,7 +1946,7 @@
         <v>7.3380999999999998</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>45708</v>
       </c>
@@ -2174,7 +1984,7 @@
         <v>7.3285999999999998</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>45709</v>
       </c>
@@ -2212,7 +2022,7 @@
         <v>7.3124000000000002</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>45712</v>
       </c>
@@ -2250,7 +2060,7 @@
         <v>7.4088000000000003</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>45713</v>
       </c>
@@ -2288,7 +2098,7 @@
         <v>7.3627000000000002</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>45714</v>
       </c>
@@ -2326,7 +2136,7 @@
         <v>7.4257999999999997</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>45715</v>
       </c>
@@ -2364,7 +2174,7 @@
         <v>7.4863999999999997</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>45716</v>
       </c>
@@ -2402,17 +2212,17 @@
         <v>7.5185000000000004</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45719</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>45720</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>45721</v>
       </c>
@@ -2450,7 +2260,7 @@
         <v>7.45</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>45722</v>
       </c>
@@ -2488,7 +2298,7 @@
         <v>7.46</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>45723</v>
       </c>
@@ -2526,7 +2336,7 @@
         <v>7.4450000000000003</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>45726</v>
       </c>
@@ -2564,7 +2374,7 @@
         <v>7.4413999999999998</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>45727</v>
       </c>
@@ -2602,7 +2412,7 @@
         <v>7.42</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>45728</v>
       </c>
@@ -2640,7 +2450,7 @@
         <v>7.4675000000000002</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>45729</v>
       </c>
@@ -2678,7 +2488,7 @@
         <v>7.4409000000000001</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>45730</v>
       </c>
@@ -2716,7 +2526,7 @@
         <v>7.4497</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>45733</v>
       </c>
@@ -2754,7 +2564,7 @@
         <v>7.4622000000000002</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>45734</v>
       </c>
@@ -2792,7 +2602,7 @@
         <v>7.4263000000000003</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>45735</v>
       </c>
@@ -2830,7 +2640,7 @@
         <v>7.37</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>45736</v>
       </c>
@@ -2868,7 +2678,7 @@
         <v>7.4149000000000003</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>45737</v>
       </c>
@@ -2906,7 +2716,7 @@
         <v>7.4</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>45740</v>
       </c>
@@ -2944,7 +2754,7 @@
         <v>7.4462000000000002</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>45741</v>
       </c>
@@ -2982,7 +2792,7 @@
         <v>7.4295</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>45742</v>
       </c>
@@ -3020,7 +2830,7 @@
         <v>7.4358000000000004</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>45743</v>
       </c>
@@ -3058,7 +2868,7 @@
         <v>7.4353999999999996</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>45744</v>
       </c>
@@ -3096,7 +2906,7 @@
         <v>7.4352999999999998</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>45747</v>
       </c>
@@ -3134,7 +2944,7 @@
         <v>7.3903999999999996</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>45748</v>
       </c>
@@ -3172,7 +2982,7 @@
         <v>7.4127999999999998</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>45749</v>
       </c>
@@ -3210,7 +3020,7 @@
         <v>7.4168000000000003</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>45750</v>
       </c>
@@ -3248,7 +3058,7 @@
         <v>7.2930999999999999</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>45751</v>
       </c>
@@ -3286,7 +3096,7 @@
         <v>7.2838000000000003</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>45754</v>
       </c>
@@ -3324,7 +3134,7 @@
         <v>7.3330000000000002</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>45755</v>
       </c>
@@ -3362,7 +3172,7 @@
         <v>7.3746</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>45756</v>
       </c>
@@ -3400,7 +3210,7 @@
         <v>7.3754999999999997</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>45757</v>
       </c>
@@ -3438,7 +3248,7 @@
         <v>7.4169999999999998</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>45758</v>
       </c>
@@ -3476,7 +3286,7 @@
         <v>7.32</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>45761</v>
       </c>
@@ -3514,7 +3324,7 @@
         <v>7.3009000000000004</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>45762</v>
       </c>
@@ -3552,7 +3362,7 @@
         <v>7.3554000000000004</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>45763</v>
       </c>
@@ -3590,7 +3400,7 @@
         <v>7.3998999999999997</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>45764</v>
       </c>
@@ -3628,17 +3438,17 @@
         <v>7.4032999999999998</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>45765</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>45768</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>45769</v>
       </c>
@@ -3676,7 +3486,7 @@
         <v>7.4922000000000004</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>45770</v>
       </c>
@@ -3714,7 +3524,7 @@
         <v>7.4551999999999996</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>45771</v>
       </c>
@@ -3752,7 +3562,7 @@
         <v>7.3647</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>45772</v>
       </c>
@@ -3790,7 +3600,7 @@
         <v>7.3592000000000004</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>45775</v>
       </c>
@@ -3828,7 +3638,7 @@
         <v>7.3460999999999999</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>45776</v>
       </c>
@@ -3866,7 +3676,7 @@
         <v>7.34</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>45777</v>
       </c>
@@ -3904,12 +3714,12 @@
         <v>7.3209999999999997</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>45778</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>45779</v>
       </c>
@@ -3947,7 +3757,7 @@
         <v>7.3235999999999999</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>45782</v>
       </c>
@@ -3985,7 +3795,7 @@
         <v>7.3532999999999999</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>45783</v>
       </c>
@@ -4023,7 +3833,7 @@
         <v>7.2789000000000001</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>45784</v>
       </c>
@@ -4061,7 +3871,7 @@
         <v>7.2285000000000004</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>45785</v>
       </c>
@@ -4099,7 +3909,7 @@
         <v>7.1429</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>45786</v>
       </c>
@@ -4137,7 +3947,7 @@
         <v>7.0960999999999999</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>45789</v>
       </c>
@@ -4175,7 +3985,7 @@
         <v>7.1116999999999999</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>45790</v>
       </c>
@@ -4213,7 +4023,7 @@
         <v>7.1037999999999997</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>45791</v>
       </c>
@@ -4251,7 +4061,7 @@
         <v>7.1600999999999999</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>45792</v>
       </c>
@@ -4289,7 +4099,7 @@
         <v>7.1432000000000002</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>45793</v>
       </c>
@@ -4327,7 +4137,7 @@
         <v>7.1170999999999998</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>45796</v>
       </c>
@@ -4365,7 +4175,7 @@
         <v>7.0759999999999996</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>45797</v>
       </c>
@@ -4403,7 +4213,7 @@
         <v>7.1161000000000003</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>45798</v>
       </c>
@@ -4441,7 +4251,7 @@
         <v>7.1333000000000002</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>45799</v>
       </c>
@@ -4479,7 +4289,7 @@
         <v>7.0876999999999999</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>45800</v>
       </c>
@@ -4517,7 +4327,7 @@
         <v>7.0891999999999999</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>45803</v>
       </c>
@@ -4555,7 +4365,7 @@
         <v>7.0759999999999996</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>45804</v>
       </c>
@@ -4593,7 +4403,7 @@
         <v>7.0393999999999997</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>45805</v>
       </c>
@@ -4631,7 +4441,7 @@
         <v>7.0735999999999999</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>45806</v>
       </c>
@@ -4669,7 +4479,7 @@
         <v>7.077</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>45807</v>
       </c>
@@ -4707,7 +4517,7 @@
         <v>7.1158999999999999</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>45810</v>
       </c>
@@ -4745,7 +4555,7 @@
         <v>7.15</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>45811</v>
       </c>
@@ -4783,7 +4593,7 @@
         <v>7.1532999999999998</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
         <v>45812</v>
       </c>
@@ -4821,7 +4631,7 @@
         <v>7.1313000000000004</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>45813</v>
       </c>
@@ -4859,7 +4669,7 @@
         <v>7.1519000000000004</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>45814</v>
       </c>
@@ -4897,7 +4707,7 @@
         <v>7.157</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>45817</v>
       </c>
@@ -4935,7 +4745,7 @@
         <v>7.1835000000000004</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>45818</v>
       </c>
@@ -4973,7 +4783,7 @@
         <v>7.2187000000000001</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>45819</v>
       </c>
@@ -5011,7 +4821,7 @@
         <v>7.1904000000000003</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>45820</v>
       </c>
@@ -5049,7 +4859,7 @@
         <v>7.1929999999999996</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>45821</v>
       </c>
@@ -5087,7 +4897,7 @@
         <v>7.17</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>45824</v>
       </c>
@@ -5125,7 +4935,7 @@
         <v>7.1406999999999998</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>45825</v>
       </c>
@@ -5163,7 +4973,7 @@
         <v>7.1124999999999998</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>45826</v>
       </c>
@@ -5201,12 +5011,12 @@
         <v>7.0688000000000004</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>45827</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
         <v>45828</v>
       </c>
@@ -5244,7 +5054,7 @@
         <v>7.0031999999999996</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>45831</v>
       </c>
@@ -5282,7 +5092,7 @@
         <v>7.0294999999999996</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>45832</v>
       </c>
@@ -5320,7 +5130,7 @@
         <v>7.0978000000000003</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>45833</v>
       </c>
@@ -5358,7 +5168,7 @@
         <v>7.1234000000000002</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>45834</v>
       </c>
@@ -5396,7 +5206,7 @@
         <v>7.0848000000000004</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>45835</v>
       </c>
@@ -5434,7 +5244,7 @@
         <v>7.0435999999999996</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>45838</v>
       </c>
@@ -5472,7 +5282,7 @@
         <v>6.9676</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="1">
         <v>45839</v>
       </c>
@@ -5510,7 +5320,7 @@
         <v>6.9507000000000003</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>45840</v>
       </c>
@@ -5548,7 +5358,7 @@
         <v>6.99</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
         <v>45841</v>
       </c>
@@ -5586,7 +5396,7 @@
         <v>6.9894999999999996</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
         <v>45842</v>
       </c>
@@ -5624,7 +5434,7 @@
         <v>6.9901999999999997</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
         <v>45845</v>
       </c>
@@ -5662,7 +5472,7 @@
         <v>7.0197000000000003</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
         <v>45846</v>
       </c>
@@ -5700,7 +5510,7 @@
         <v>7.0736999999999997</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
         <v>45847</v>
       </c>
@@ -5738,7 +5548,7 @@
         <v>7.0975999999999999</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
         <v>45848</v>
       </c>
@@ -5776,7 +5586,7 @@
         <v>7.1064999999999996</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="1">
         <v>45849</v>
       </c>
@@ -5814,7 +5624,7 @@
         <v>7.0709</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="1">
         <v>45852</v>
       </c>
@@ -5852,7 +5662,7 @@
         <v>7.1104000000000003</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
         <v>45853</v>
       </c>
@@ -5890,7 +5700,7 @@
         <v>7.1527000000000003</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
         <v>45854</v>
       </c>
@@ -5928,7 +5738,7 @@
         <v>7.21</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="1">
         <v>45855</v>
       </c>
@@ -5966,7 +5776,7 @@
         <v>7.1784999999999997</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
         <v>45856</v>
       </c>
@@ -6004,7 +5814,7 @@
         <v>7.2046000000000001</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
         <v>45859</v>
       </c>
@@ -6042,7 +5852,7 @@
         <v>7.2096999999999998</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A147" s="1">
         <v>45860</v>
       </c>
@@ -6080,7 +5890,7 @@
         <v>7.2275999999999998</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A148" s="1">
         <v>45861</v>
       </c>
@@ -6118,7 +5928,7 @@
         <v>7.1965000000000003</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A149" s="1">
         <v>45862</v>
       </c>
@@ -6156,7 +5966,7 @@
         <v>7.1989000000000001</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A150" s="1">
         <v>45863</v>
       </c>
@@ -6194,7 +6004,7 @@
         <v>7.2237999999999998</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A151" s="1">
         <v>45866</v>
       </c>
@@ -6232,7 +6042,7 @@
         <v>7.22</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>45867</v>
       </c>
@@ -6270,7 +6080,7 @@
         <v>7.1798000000000002</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A153" s="1">
         <v>45868</v>
       </c>
@@ -6308,7 +6118,7 @@
         <v>7.18</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
         <v>45869</v>
       </c>
@@ -6346,7 +6156,7 @@
         <v>7.1835000000000004</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A155" s="1">
         <v>45870</v>
       </c>
@@ -6384,7 +6194,7 @@
         <v>7.1699000000000002</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A156" s="1">
         <v>45873</v>
       </c>
@@ -6422,7 +6232,7 @@
         <v>7.1733000000000002</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A157" s="1">
         <v>45874</v>
       </c>
@@ -6460,7 +6270,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A158" s="1">
         <v>45875</v>
       </c>
@@ -6498,7 +6308,7 @@
         <v>7.1971999999999996</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A159" s="1">
         <v>45876</v>
       </c>
@@ -6536,7 +6346,7 @@
         <v>7.13</v>
       </c>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A160" s="1">
         <v>45877</v>
       </c>
@@ -6574,7 +6384,7 @@
         <v>7.15</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
         <v>45880</v>
       </c>
@@ -6612,7 +6422,7 @@
         <v>7.1353</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A162" s="1">
         <v>45881</v>
       </c>
@@ -6650,7 +6460,7 @@
         <v>7.1483999999999996</v>
       </c>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A163" s="1">
         <v>45882</v>
       </c>
@@ -6688,7 +6498,7 @@
         <v>7.15</v>
       </c>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A164" s="1">
         <v>45883</v>
       </c>
@@ -6726,7 +6536,7 @@
         <v>7.1428000000000003</v>
       </c>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A165" s="1">
         <v>45884</v>
       </c>
@@ -6764,7 +6574,7 @@
         <v>7.1325000000000003</v>
       </c>
     </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A166" s="1">
         <v>45887</v>
       </c>
@@ -6802,7 +6612,7 @@
         <v>7.1608999999999998</v>
       </c>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A167" s="1">
         <v>45888</v>
       </c>
@@ -6840,7 +6650,7 @@
         <v>7.2839999999999998</v>
       </c>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A168" s="1">
         <v>45889</v>
       </c>
@@ -6878,7 +6688,7 @@
         <v>7.3087</v>
       </c>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A169" s="1">
         <v>45890</v>
       </c>
@@ -6916,7 +6726,7 @@
         <v>7.33</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A170" s="1">
         <v>45891</v>
       </c>
@@ -6954,7 +6764,7 @@
         <v>7.2731000000000003</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A171" s="1">
         <v>45894</v>
       </c>
@@ -6992,7 +6802,7 @@
         <v>7.2252000000000001</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A172" s="1">
         <v>45895</v>
       </c>
@@ -7030,7 +6840,7 @@
         <v>7.22</v>
       </c>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A173" s="1">
         <v>45896</v>
       </c>
@@ -7068,7 +6878,7 @@
         <v>7.2224000000000004</v>
       </c>
     </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A174" s="1">
         <v>45897</v>
       </c>
@@ -7106,7 +6916,7 @@
         <v>7.19</v>
       </c>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A175" s="1">
         <v>45898</v>
       </c>
@@ -7144,7 +6954,7 @@
         <v>7.2249999999999996</v>
       </c>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A176" s="1">
         <v>45901</v>
       </c>
@@ -7182,7 +6992,7 @@
         <v>7.2857000000000003</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A177" s="1">
         <v>45902</v>
       </c>
@@ -7220,7 +7030,7 @@
         <v>7.3</v>
       </c>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A178" s="1">
         <v>45903</v>
       </c>
@@ -7258,7 +7068,7 @@
         <v>7.36</v>
       </c>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A179" s="1">
         <v>45904</v>
       </c>
@@ -7296,7 +7106,7 @@
         <v>7.3787000000000003</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A180" s="1">
         <v>45905</v>
       </c>
@@ -7334,7 +7144,7 @@
         <v>7.3410000000000002</v>
       </c>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A181" s="1">
         <v>45908</v>
       </c>
@@ -7372,7 +7182,7 @@
         <v>7.3056000000000001</v>
       </c>
     </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A182" s="1">
         <v>45909</v>
       </c>
@@ -7410,7 +7220,7 @@
         <v>7.2946999999999997</v>
       </c>
     </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A183" s="1">
         <v>45910</v>
       </c>
@@ -7448,7 +7258,7 @@
         <v>7.26</v>
       </c>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A184" s="1">
         <v>45911</v>
       </c>
@@ -7486,7 +7296,7 @@
         <v>7.2361000000000004</v>
       </c>
     </row>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A185" s="1">
         <v>45912</v>
       </c>
@@ -7524,7 +7334,7 @@
         <v>7.2262000000000004</v>
       </c>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A186" s="1">
         <v>45915</v>
       </c>
@@ -7562,7 +7372,7 @@
         <v>7.21</v>
       </c>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A187" s="1">
         <v>45916</v>
       </c>
@@ -7600,7 +7410,7 @@
         <v>7.1649000000000003</v>
       </c>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A188" s="1">
         <v>45917</v>
       </c>
@@ -7638,7 +7448,7 @@
         <v>7.15</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A189" s="1">
         <v>45918</v>
       </c>
@@ -7676,7 +7486,7 @@
         <v>7.18</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A190" s="1">
         <v>45919</v>
       </c>
@@ -7714,7 +7524,7 @@
         <v>7.2172000000000001</v>
       </c>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A191" s="1">
         <v>45922</v>
       </c>
@@ -7752,7 +7562,7 @@
         <v>7.26</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A192" s="1">
         <v>45923</v>
       </c>
@@ -7790,7 +7600,7 @@
         <v>7.23</v>
       </c>
     </row>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A193" s="1">
         <v>45924</v>
       </c>
@@ -7828,7 +7638,7 @@
         <v>7.22</v>
       </c>
     </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A194" s="1">
         <v>45925</v>
       </c>
@@ -7866,7 +7676,7 @@
         <v>7.22</v>
       </c>
     </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A195" s="1">
         <v>45926</v>
       </c>
@@ -7904,7 +7714,7 @@
         <v>7.21</v>
       </c>
     </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A196" s="1">
         <v>45929</v>
       </c>
@@ -7942,7 +7752,7 @@
         <v>7.2405999999999997</v>
       </c>
     </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A197" s="1">
         <v>45930</v>
       </c>
@@ -7980,7 +7790,7 @@
         <v>7.2446999999999999</v>
       </c>
     </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A198" s="1">
         <v>45931</v>
       </c>
@@ -8018,7 +7828,7 @@
         <v>7.2309999999999999</v>
       </c>
     </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A199" s="1">
         <v>45932</v>
       </c>
@@ -8056,7 +7866,7 @@
         <v>7.2678000000000003</v>
       </c>
     </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A200" s="1">
         <v>45933</v>
       </c>
@@ -8094,7 +7904,7 @@
         <v>7.2723000000000004</v>
       </c>
     </row>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A201" s="1">
         <v>45936</v>
       </c>
@@ -8132,7 +7942,7 @@
         <v>7.2773000000000003</v>
       </c>
     </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A202" s="1">
         <v>45937</v>
       </c>
@@ -8170,7 +7980,7 @@
         <v>7.3158000000000003</v>
       </c>
     </row>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A203" s="1">
         <v>45938</v>
       </c>
@@ -8208,7 +8018,7 @@
         <v>7.32</v>
       </c>
     </row>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A204" s="1">
         <v>45939</v>
       </c>
@@ -8246,7 +8056,7 @@
         <v>7.3120000000000003</v>
       </c>
     </row>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A205" s="1">
         <v>45940</v>
       </c>
@@ -8292,12 +8102,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{758C3EF2-6C72-45F1-A0D5-5BC47AE03FB1}">
   <dimension ref="A1:L205"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -8335,7 +8145,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -8373,53 +8183,53 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="2">
-        <f>_xll.ECONOMATICA(B1,"CLOSE",,"D-0","2025-01-01","D",,,,"FALSE",,)</f>
-        <v>45658</v>
-      </c>
-      <c r="C3" t="str">
-        <f>_xll.ECONOMATICA(C1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <f>_xll.ECONOMATICA(D1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <f>_xll.ECONOMATICA(E1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <f>_xll.ECONOMATICA(F1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <f>_xll.ECONOMATICA(G1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <f>_xll.ECONOMATICA(H1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <f>_xll.ECONOMATICA(I1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <f>_xll.ECONOMATICA(J1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="K3" t="str">
-        <f>_xll.ECONOMATICA(K1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <f>_xll.ECONOMATICA(L1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="e">
+        <f ca="1">_xll.ECONOMATICA(B1,"CLOSE",,"D-0","2025-01-01","D",,,,"FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="C3" t="e">
+        <f ca="1">_xll.ECONOMATICA(C1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="D3" t="e">
+        <f ca="1">_xll.ECONOMATICA(D1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="E3" t="e">
+        <f ca="1">_xll.ECONOMATICA(E1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="F3" t="e">
+        <f ca="1">_xll.ECONOMATICA(F1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="G3" t="e">
+        <f ca="1">_xll.ECONOMATICA(G1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="H3" t="e">
+        <f ca="1">_xll.ECONOMATICA(H1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I3" t="e">
+        <f ca="1">_xll.ECONOMATICA(I1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="J3" t="e">
+        <f ca="1">_xll.ECONOMATICA(J1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="K3" t="e">
+        <f ca="1">_xll.ECONOMATICA(K1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="L3" t="e">
+        <f ca="1">_xll.ECONOMATICA(L1,"CLOSE",,"D-0","2025-01-01","D",,,"FALSE","FALSE",,)</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>45659</v>
       </c>
@@ -8457,7 +8267,7 @@
         <v>3509.3190994000001</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>45660</v>
       </c>
@@ -8495,7 +8305,7 @@
         <v>3520.4852793</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>45663</v>
       </c>
@@ -8533,7 +8343,7 @@
         <v>3543.7757267000002</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>45664</v>
       </c>
@@ -8571,7 +8381,7 @@
         <v>3546.7278338000001</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>45665</v>
       </c>
@@ -8609,7 +8419,7 @@
         <v>3552.8817911000001</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>45666</v>
       </c>
@@ -8647,7 +8457,7 @@
         <v>3548.9216271999999</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>45667</v>
       </c>
@@ -8685,7 +8495,7 @@
         <v>3527.3201906999998</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>45670</v>
       </c>
@@ -8723,7 +8533,7 @@
         <v>3511.6229011</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>45671</v>
       </c>
@@ -8761,7 +8571,7 @@
         <v>3529.7578572000002</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>45672</v>
       </c>
@@ -8799,7 +8609,7 @@
         <v>3549.6930438999998</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>45673</v>
       </c>
@@ -8837,7 +8647,7 @@
         <v>3528.2822053</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>45674</v>
       </c>
@@ -8875,7 +8685,7 @@
         <v>3494.0369799999999</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>45677</v>
       </c>
@@ -8913,7 +8723,7 @@
         <v>3473.7418438999998</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>45678</v>
       </c>
@@ -8951,7 +8761,7 @@
         <v>3453.3432965000002</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>45679</v>
       </c>
@@ -8989,7 +8799,7 @@
         <v>3459.5082680999999</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>45680</v>
       </c>
@@ -9027,7 +8837,7 @@
         <v>3444.1497260000001</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>45681</v>
       </c>
@@ -9065,7 +8875,7 @@
         <v>3450.573582</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>45684</v>
       </c>
@@ -9103,7 +8913,7 @@
         <v>3453.0303878</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>45685</v>
       </c>
@@ -9141,7 +8951,7 @@
         <v>3450.8082202999999</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>45686</v>
       </c>
@@ -9179,7 +8989,7 @@
         <v>3449.6586453999998</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>45687</v>
       </c>
@@ -9217,7 +9027,7 @@
         <v>3507.4658795999999</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>45688</v>
       </c>
@@ -9255,7 +9065,7 @@
         <v>3497.7560758999998</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>45691</v>
       </c>
@@ -9293,7 +9103,7 @@
         <v>3516.5057529000001</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>45692</v>
       </c>
@@ -9331,7 +9141,7 @@
         <v>3512.4367699999998</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>45693</v>
       </c>
@@ -9369,7 +9179,7 @@
         <v>3484.9439867000001</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>45694</v>
       </c>
@@ -9407,7 +9217,7 @@
         <v>3503.0797564999998</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>45695</v>
       </c>
@@ -9445,7 +9255,7 @@
         <v>3491.5853473000002</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>45698</v>
       </c>
@@ -9483,7 +9293,7 @@
         <v>3493.5432096999998</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>45699</v>
       </c>
@@ -9521,7 +9331,7 @@
         <v>3503.9992151000001</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>45700</v>
       </c>
@@ -9559,7 +9369,7 @@
         <v>3507.4020518000002</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>45701</v>
       </c>
@@ -9597,7 +9407,7 @@
         <v>3514.2281413000001</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>45702</v>
       </c>
@@ -9635,7 +9445,7 @@
         <v>3572.7668349</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>45705</v>
       </c>
@@ -9673,7 +9483,7 @@
         <v>3593.0652123</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>45706</v>
       </c>
@@ -9711,7 +9521,7 @@
         <v>3590.5408837999998</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>45707</v>
       </c>
@@ -9749,7 +9559,7 @@
         <v>3585.26847</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>45708</v>
       </c>
@@ -9787,7 +9597,7 @@
         <v>3593.2345911000002</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>45709</v>
       </c>
@@ -9825,7 +9635,7 @@
         <v>3604.2773275999998</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>45712</v>
       </c>
@@ -9863,7 +9673,7 @@
         <v>3564.4342188999999</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>45713</v>
       </c>
@@ -9901,7 +9711,7 @@
         <v>3588.7928388</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>45714</v>
       </c>
@@ -9939,7 +9749,7 @@
         <v>3563.4609393999999</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>45715</v>
       </c>
@@ -9977,7 +9787,7 @@
         <v>3540.1684955999999</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>45716</v>
       </c>
@@ -10015,17 +9825,17 @@
         <v>3529.6178051000002</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45719</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>45720</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>45721</v>
       </c>
@@ -10063,7 +9873,7 @@
         <v>3563.3482503</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>45722</v>
       </c>
@@ -10101,7 +9911,7 @@
         <v>3562.4656967000001</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>45723</v>
       </c>
@@ -10139,7 +9949,7 @@
         <v>3572.6875341</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>45726</v>
       </c>
@@ -10177,7 +9987,7 @@
         <v>3577.8587441</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>45727</v>
       </c>
@@ -10215,7 +10025,7 @@
         <v>3590.997304</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>45728</v>
       </c>
@@ -10253,7 +10063,7 @@
         <v>3573.9661064000002</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>45729</v>
       </c>
@@ -10291,7 +10101,7 @@
         <v>3589.4286505</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>45730</v>
       </c>
@@ -10329,7 +10139,7 @@
         <v>3589.1148978000001</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>45733</v>
       </c>
@@ -10367,7 +10177,7 @@
         <v>3587.1593149999999</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>45734</v>
       </c>
@@ -10405,7 +10215,7 @@
         <v>3605.2373398999998</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>45735</v>
       </c>
@@ -10443,7 +10253,7 @@
         <v>3632.7055624</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>45736</v>
       </c>
@@ -10481,7 +10291,7 @@
         <v>3614.4044942999999</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>45737</v>
       </c>
@@ -10519,7 +10329,7 @@
         <v>3623.1530238</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>45740</v>
       </c>
@@ -10557,7 +10367,7 @@
         <v>3604.3850461000002</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>45741</v>
       </c>
@@ -10595,7 +10405,7 @@
         <v>3613.9000117000001</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>45742</v>
       </c>
@@ -10633,7 +10443,7 @@
         <v>3613.0927830000001</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>45743</v>
       </c>
@@ -10671,7 +10481,7 @@
         <v>3615.2943312000002</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>45744</v>
       </c>
@@ -10709,7 +10519,7 @@
         <v>3616.9046165999998</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>45747</v>
       </c>
@@ -10747,7 +10557,7 @@
         <v>3639.1537715999998</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>45748</v>
       </c>
@@ -10785,7 +10595,7 @@
         <v>3630.9919762</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>45749</v>
       </c>
@@ -10823,7 +10633,7 @@
         <v>3631.1657531999999</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>45750</v>
       </c>
@@ -10861,7 +10671,7 @@
         <v>3689.7525377000002</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>45751</v>
       </c>
@@ -10899,7 +10709,7 @@
         <v>3696.0686018000001</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>45754</v>
       </c>
@@ -10937,7 +10747,7 @@
         <v>3675.3077524999999</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>45755</v>
       </c>
@@ -10975,7 +10785,7 @@
         <v>3658.2444571999999</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>45756</v>
       </c>
@@ -11013,7 +10823,7 @@
         <v>3659.8241174</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>45757</v>
       </c>
@@ -11051,7 +10861,7 @@
         <v>3642.9684351999999</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>45758</v>
       </c>
@@ -11089,7 +10899,7 @@
         <v>3689.6110847</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>45761</v>
       </c>
@@ -11127,7 +10937,7 @@
         <v>3700.4688528000001</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>45762</v>
       </c>
@@ -11165,7 +10975,7 @@
         <v>3677.3519583000002</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>45763</v>
       </c>
@@ -11203,7 +11013,7 @@
         <v>3658.8675944000001</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>45764</v>
       </c>
@@ -11241,17 +11051,17 @@
         <v>3659.1521112999999</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>45765</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>45768</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>45769</v>
       </c>
@@ -11289,7 +11099,7 @@
         <v>3621.0018381999998</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>45770</v>
       </c>
@@ -11327,7 +11137,7 @@
         <v>3639.3639643000001</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>45771</v>
       </c>
@@ -11365,7 +11175,7 @@
         <v>3682.2344290999999</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>45772</v>
       </c>
@@ -11403,7 +11213,7 @@
         <v>3686.5897570000002</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>45775</v>
       </c>
@@ -11441,7 +11251,7 @@
         <v>3694.5758639000001</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>45776</v>
       </c>
@@ -11479,7 +11289,7 @@
         <v>3699.2417578</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>45777</v>
       </c>
@@ -11517,12 +11327,12 @@
         <v>3709.8739660000001</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>45778</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>45779</v>
       </c>
@@ -11560,7 +11370,7 @@
         <v>3710.5271840999999</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>45782</v>
       </c>
@@ -11598,7 +11408,7 @@
         <v>3698.6896827</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>45783</v>
       </c>
@@ -11636,7 +11446,7 @@
         <v>3735.0419059000001</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>45784</v>
       </c>
@@ -11674,7 +11484,7 @@
         <v>3760.5975204000001</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>45785</v>
       </c>
@@ -11712,7 +11522,7 @@
         <v>3803.324376</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>45786</v>
       </c>
@@ -11750,7 +11560,7 @@
         <v>3828.1816125999999</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>45789</v>
       </c>
@@ -11788,7 +11598,7 @@
         <v>3822.5017914999999</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>45790</v>
       </c>
@@ -11826,7 +11636,7 @@
         <v>3828.2475792999999</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>45791</v>
       </c>
@@ -11864,7 +11674,7 @@
         <v>3802.9396462999998</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>45792</v>
       </c>
@@ -11902,7 +11712,7 @@
         <v>3812.9751559000001</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>45793</v>
       </c>
@@ -11940,7 +11750,7 @@
         <v>3827.2864202000001</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>45796</v>
       </c>
@@ -11978,7 +11788,7 @@
         <v>3849.0079093999998</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>45797</v>
       </c>
@@ -12016,7 +11826,7 @@
         <v>3831.1480778999999</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>45798</v>
       </c>
@@ -12054,7 +11864,7 @@
         <v>3824.5009853000001</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>45799</v>
       </c>
@@ -12092,7 +11902,7 @@
         <v>3848.360768</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>45800</v>
       </c>
@@ -12130,7 +11940,7 @@
         <v>3849.3165319999998</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>45803</v>
       </c>
@@ -12168,7 +11978,7 @@
         <v>3857.4704949000002</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>45804</v>
       </c>
@@ -12206,7 +12016,7 @@
         <v>3877.1763391999998</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>45805</v>
       </c>
@@ -12244,7 +12054,7 @@
         <v>3861.5664683999998</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>45806</v>
       </c>
@@ -12282,7 +12092,7 @@
         <v>3861.5425986</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>45807</v>
       </c>
@@ -12320,7 +12130,7 @@
         <v>3844.1995259</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>45810</v>
       </c>
@@ -12358,7 +12168,7 @@
         <v>3829.3305381</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>45811</v>
       </c>
@@ -12396,7 +12206,7 @@
         <v>3829.3799957000001</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
         <v>45812</v>
       </c>
@@ -12434,7 +12244,7 @@
         <v>3841.6561784</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>45813</v>
       </c>
@@ -12472,7 +12282,7 @@
         <v>3833.3394557000001</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>45814</v>
       </c>
@@ -12510,7 +12320,7 @@
         <v>3832.5244060999999</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>45817</v>
       </c>
@@ -12548,7 +12358,7 @@
         <v>3821.4293782</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>45818</v>
       </c>
@@ -12586,7 +12396,7 @@
         <v>3803.7889621999998</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>45819</v>
       </c>
@@ -12624,7 +12434,7 @@
         <v>3818.7803281000001</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>45820</v>
       </c>
@@ -12662,7 +12472,7 @@
         <v>3819.0389294000001</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>45821</v>
       </c>
@@ -12700,7 +12510,7 @@
         <v>3831.5675486999999</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>45824</v>
       </c>
@@ -12738,7 +12548,7 @@
         <v>3847.1964259000001</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>45825</v>
       </c>
@@ -12776,7 +12586,7 @@
         <v>3862.4288504000001</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>45826</v>
       </c>
@@ -12814,12 +12624,12 @@
         <v>3885.3603085</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>45827</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
         <v>45828</v>
       </c>
@@ -12857,7 +12667,7 @@
         <v>3919.3982780000001</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>45831</v>
       </c>
@@ -12895,7 +12705,7 @@
         <v>3907.8784778999998</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>45832</v>
       </c>
@@ -12933,7 +12743,7 @@
         <v>3875.8228789999998</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>45833</v>
       </c>
@@ -12971,7 +12781,7 @@
         <v>3864.9107531999998</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>45834</v>
       </c>
@@ -13009,7 +12819,7 @@
         <v>3885.2991307000002</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>45835</v>
       </c>
@@ -13047,7 +12857,7 @@
         <v>3906.0532352</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>45838</v>
       </c>
@@ -13085,7 +12895,7 @@
         <v>3945.3729156999998</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="1">
         <v>45839</v>
       </c>
@@ -13123,7 +12933,7 @@
         <v>3955.3150105</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>45840</v>
       </c>
@@ -13161,7 +12971,7 @@
         <v>3936.9950597000002</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
         <v>45841</v>
       </c>
@@ -13199,7 +13009,7 @@
         <v>3938.6764428000001</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
         <v>45842</v>
       </c>
@@ -13237,7 +13047,7 @@
         <v>3939.7544968000002</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
         <v>45845</v>
       </c>
@@ -13275,7 +13085,7 @@
         <v>3926.4670882999999</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
         <v>45846</v>
       </c>
@@ -13313,7 +13123,7 @@
         <v>3901.2075445999999</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
         <v>45847</v>
       </c>
@@ -13351,7 +13161,7 @@
         <v>3890.9196892</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
         <v>45848</v>
       </c>
@@ -13389,7 +13199,7 @@
         <v>3889.6524717000002</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="1">
         <v>45849</v>
       </c>
@@ -13427,7 +13237,7 @@
         <v>3908.6247714000001</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="1">
         <v>45852</v>
       </c>
@@ -13465,7 +13275,7 @@
         <v>3890.8039583999998</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
         <v>45853</v>
       </c>
@@ -13503,7 +13313,7 @@
         <v>3871.7920785000001</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
         <v>45854</v>
       </c>
@@ -13541,7 +13351,7 @@
         <v>3845.9176941000001</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="1">
         <v>45855</v>
       </c>
@@ -13579,7 +13389,7 @@
         <v>3862.6570198999998</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
         <v>45856</v>
       </c>
@@ -13617,7 +13427,7 @@
         <v>3851.7916291000001</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
         <v>45859</v>
       </c>
@@ -13655,7 +13465,7 @@
         <v>3851.0052989999999</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A147" s="1">
         <v>45860</v>
       </c>
@@ -13693,7 +13503,7 @@
         <v>3844.1226753000001</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A148" s="1">
         <v>45861</v>
       </c>
@@ -13731,7 +13541,7 @@
         <v>3860.6173273999998</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A149" s="1">
         <v>45862</v>
       </c>
@@ -13769,7 +13579,7 @@
         <v>3861.1205395000002</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A150" s="1">
         <v>45863</v>
       </c>
@@ -13807,7 +13617,7 @@
         <v>3850.8819570999999</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A151" s="1">
         <v>45866</v>
       </c>
@@ -13845,7 +13655,7 @@
         <v>3854.4938989000002</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>45867</v>
       </c>
@@ -13883,7 +13693,7 @@
         <v>3875.4163011999999</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A153" s="1">
         <v>45868</v>
       </c>
@@ -13921,7 +13731,7 @@
         <v>3876.9912943999998</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
         <v>45869</v>
       </c>
@@ -13959,7 +13769,7 @@
         <v>3876.9784728999998</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A155" s="1">
         <v>45870</v>
       </c>
@@ -13997,7 +13807,7 @@
         <v>3885.2018475</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A156" s="1">
         <v>45873</v>
       </c>
@@ -14035,7 +13845,7 @@
         <v>3885.2383918</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A157" s="1">
         <v>45874</v>
       </c>
@@ -14073,7 +13883,7 @@
         <v>3874.0819268</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A158" s="1">
         <v>45875</v>
       </c>
@@ -14111,7 +13921,7 @@
         <v>3877.0974108</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A159" s="1">
         <v>45876</v>
       </c>
@@ -14149,7 +13959,7 @@
         <v>3911.2441884</v>
       </c>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A160" s="1">
         <v>45877</v>
       </c>
@@ -14187,7 +13997,7 @@
         <v>3903.2085861</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
         <v>45880</v>
       </c>
@@ -14225,7 +14035,7 @@
         <v>3912.0273578000001</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A162" s="1">
         <v>45881</v>
       </c>
@@ -14263,7 +14073,7 @@
         <v>3903.9578372000001</v>
       </c>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A163" s="1">
         <v>45882</v>
       </c>
@@ -14301,7 +14111,7 @@
         <v>3904.6926164000001</v>
       </c>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A164" s="1">
         <v>45883</v>
       </c>
@@ -14339,7 +14149,7 @@
         <v>3909.6989773</v>
       </c>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A165" s="1">
         <v>45884</v>
       </c>
@@ -14377,7 +14187,7 @@
         <v>3916.2123999999999</v>
       </c>
     </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A166" s="1">
         <v>45887</v>
       </c>
@@ -14415,7 +14225,7 @@
         <v>3902.815818</v>
       </c>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A167" s="1">
         <v>45888</v>
       </c>
@@ -14453,7 +14263,7 @@
         <v>3842.9489939999999</v>
       </c>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A168" s="1">
         <v>45889</v>
       </c>
@@ -14491,7 +14301,7 @@
         <v>3831.8191339999998</v>
       </c>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A169" s="1">
         <v>45890</v>
       </c>
@@ -14529,7 +14339,7 @@
         <v>3822.388477</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A170" s="1">
         <v>45891</v>
       </c>
@@ -14567,7 +14377,7 @@
         <v>3850.8199519999998</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A171" s="1">
         <v>45894</v>
       </c>
@@ -14605,7 +14415,7 @@
         <v>3875.1490530000001</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A172" s="1">
         <v>45895</v>
       </c>
@@ -14643,7 +14453,7 @@
         <v>3878.5679089999999</v>
       </c>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A173" s="1">
         <v>45896</v>
       </c>
@@ -14681,7 +14491,7 @@
         <v>3878.0847530000001</v>
       </c>
     </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A174" s="1">
         <v>45897</v>
       </c>
@@ -14719,7 +14529,7 @@
         <v>3894.9454609999998</v>
       </c>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A175" s="1">
         <v>45898</v>
       </c>
@@ -14757,7 +14567,7 @@
         <v>3878.4711189999998</v>
       </c>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A176" s="1">
         <v>45901</v>
       </c>
@@ -14795,7 +14605,7 @@
         <v>3849.6012569999998</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A177" s="1">
         <v>45902</v>
       </c>
@@ -14833,7 +14643,7 @@
         <v>3843.5001950000001</v>
       </c>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A178" s="1">
         <v>45903</v>
       </c>
@@ -14871,7 +14681,7 @@
         <v>3815.4527670000002</v>
       </c>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A179" s="1">
         <v>45904</v>
       </c>
@@ -14909,7 +14719,7 @@
         <v>3807.3673159999998</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A180" s="1">
         <v>45905</v>
       </c>
@@ -14947,7 +14757,7 @@
         <v>3826.2358429999999</v>
       </c>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A181" s="1">
         <v>45908</v>
       </c>
@@ -14985,7 +14795,7 @@
         <v>3844.1357440000002</v>
       </c>
     </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A182" s="1">
         <v>45909</v>
       </c>
@@ -15023,7 +14833,7 @@
         <v>3850.2528630000002</v>
       </c>
     </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A183" s="1">
         <v>45910</v>
       </c>
@@ -15061,7 +14871,7 @@
         <v>3868.6384159999998</v>
       </c>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A184" s="1">
         <v>45911</v>
       </c>
@@ -15099,7 +14909,7 @@
         <v>3881.2238600000001</v>
       </c>
     </row>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A185" s="1">
         <v>45912</v>
       </c>
@@ -15137,7 +14947,7 @@
         <v>3886.9627949999999</v>
       </c>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A186" s="1">
         <v>45915</v>
       </c>
@@ -15175,7 +14985,7 @@
         <v>3895.8218849999998</v>
       </c>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A187" s="1">
         <v>45916</v>
       </c>
@@ -15213,7 +15023,7 @@
         <v>3920.3656150000002</v>
       </c>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A188" s="1">
         <v>45917</v>
       </c>
@@ -15251,7 +15061,7 @@
         <v>3929.977324</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A189" s="1">
         <v>45918</v>
       </c>
@@ -15289,7 +15099,7 @@
         <v>3917.1630960000002</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A190" s="1">
         <v>45919</v>
       </c>
@@ -15327,7 +15137,7 @@
         <v>3900.8857710000002</v>
       </c>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A191" s="1">
         <v>45922</v>
       </c>
@@ -15365,7 +15175,7 @@
         <v>3882.0100520000001</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A192" s="1">
         <v>45923</v>
       </c>
@@ -15403,7 +15213,7 @@
         <v>3898.8902320000002</v>
       </c>
     </row>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A193" s="1">
         <v>45924</v>
       </c>
@@ -15441,7 +15251,7 @@
         <v>3905.9809</v>
       </c>
     </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A194" s="1">
         <v>45925</v>
       </c>
@@ -15479,7 +15289,7 @@
         <v>3908.142738</v>
       </c>
     </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A195" s="1">
         <v>45926</v>
       </c>
@@ -15517,7 +15327,7 @@
         <v>3914.1337669999998</v>
       </c>
     </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A196" s="1">
         <v>45929</v>
       </c>
@@ -15555,7 +15365,7 @@
         <v>3901.0778369999998</v>
       </c>
     </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A197" s="1">
         <v>45930</v>
       </c>
@@ -15593,7 +15403,7 @@
         <v>3901.0959809999999</v>
       </c>
     </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A198" s="1">
         <v>45931</v>
       </c>
@@ -15631,7 +15441,7 @@
         <v>3909.880478</v>
       </c>
     </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A199" s="1">
         <v>45932</v>
       </c>
@@ -15669,7 +15479,7 @@
         <v>3893.8463160000001</v>
       </c>
     </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A200" s="1">
         <v>45933</v>
       </c>
@@ -15707,7 +15517,7 @@
         <v>3893.6844890000002</v>
       </c>
     </row>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A201" s="1">
         <v>45936</v>
       </c>
@@ -15745,7 +15555,7 @@
         <v>3893.281058</v>
       </c>
     </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A202" s="1">
         <v>45937</v>
       </c>
@@ -15783,7 +15593,7 @@
         <v>3876.588264</v>
       </c>
     </row>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A203" s="1">
         <v>45938</v>
       </c>
@@ -15821,7 +15631,7 @@
         <v>3876.5899239999999</v>
       </c>
     </row>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A204" s="1">
         <v>45939</v>
       </c>
@@ -15859,7 +15669,7 @@
         <v>3880.6071959999999</v>
       </c>
     </row>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A205" s="1">
         <v>45940</v>
       </c>

</xml_diff>